<commit_message>
Refresh gap matrix for conversation history features
</commit_message>
<xml_diff>
--- a/docs/HermanPrompt_Gap_Matrix.xlsx
+++ b/docs/HermanPrompt_Gap_Matrix.xlsx
@@ -832,9 +832,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:ns3="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
@@ -844,7 +844,7 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15" ns3:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -864,7 +864,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -884,7 +884,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -904,7 +904,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ns3:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>16</v>
       </c>
@@ -924,7 +924,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="48" ns3:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>19</v>
       </c>
@@ -944,7 +944,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ns3:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -964,7 +964,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>30</v>
       </c>
@@ -984,7 +984,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ns3:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>33</v>
       </c>
@@ -1004,7 +1004,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ns3:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>35</v>
       </c>
@@ -1024,7 +1024,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -1044,127 +1044,175 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>Aligned</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>Aligned</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D13" s="1" t="inlineStr">
+        <is>
+          <t>Aligned</t>
+        </is>
+      </c>
+      <c r="E13" s="1" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="F13" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>Aligned</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>Delete implemented; rename/archive not implemented</t>
+        </is>
+      </c>
+      <c r="D15" s="1" t="inlineStr">
+        <is>
+          <t>Partial gap</t>
+        </is>
+      </c>
+      <c r="E15" s="1" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="F15" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ns3:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F16" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>Plain-text export implemented; PDF not implemented</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>Partial gap</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>53</v>
       </c>
@@ -1184,7 +1232,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ns3:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>57</v>
       </c>
@@ -1204,7 +1252,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ns3:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>60</v>
       </c>
@@ -1224,7 +1272,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>62</v>
       </c>
@@ -1244,7 +1292,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>65</v>
       </c>
@@ -1264,7 +1312,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>67</v>
       </c>
@@ -1284,7 +1332,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>69</v>
       </c>
@@ -1304,7 +1352,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ns3:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>72</v>
       </c>
@@ -1324,7 +1372,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>74</v>
       </c>
@@ -1344,7 +1392,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ns3:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>78</v>
       </c>
@@ -1364,7 +1412,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" ns3:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>80</v>
       </c>
@@ -1384,7 +1432,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>82</v>
       </c>
@@ -1404,7 +1452,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ns3:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>85</v>
       </c>
@@ -1424,7 +1472,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>87</v>
       </c>
@@ -1444,7 +1492,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>89</v>
       </c>
@@ -1464,7 +1512,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ns3:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>93</v>
       </c>
@@ -1484,7 +1532,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>95</v>
       </c>
@@ -1504,7 +1552,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" ns3:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>97</v>
       </c>
@@ -1524,7 +1572,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ns3:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>99</v>
       </c>
@@ -1544,7 +1592,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>102</v>
       </c>
@@ -1564,7 +1612,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>104</v>
       </c>
@@ -1584,7 +1632,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>106</v>
       </c>
@@ -1604,7 +1652,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ns3:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>108</v>
       </c>
@@ -1624,7 +1672,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ns3:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>110</v>
       </c>
@@ -1644,27 +1692,35 @@
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" ht="48" ns3:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>112</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>Feedback plus conversations and turns are persisted; broader platform tables are still missing</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>Partial gap</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>Phase 2-5</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ns3:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>116</v>
       </c>
@@ -1684,7 +1740,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>120</v>
       </c>
@@ -1704,7 +1760,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>124</v>
       </c>
@@ -1724,7 +1780,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>128</v>
       </c>
@@ -1744,7 +1800,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>131</v>
       </c>
@@ -1764,7 +1820,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>133</v>
       </c>
@@ -1784,7 +1840,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" ht="32" ns3:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>137</v>
       </c>

</xml_diff>